<commit_message>
Testing For Print Issues
</commit_message>
<xml_diff>
--- a/Excel/car inventory.xlsx
+++ b/Excel/car inventory.xlsx
@@ -1,21 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\j-l-data-science-data-analytics\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Tests\j-l-data-science-data-analytics\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9258AC24-450D-42FD-979D-3BC647337D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB915F5-6497-48D7-AF85-94076CAE0544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{6F1C8A56-E294-480C-BFA2-897A20BA14D1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6F1C8A56-E294-480C-BFA2-897A20BA14D1}"/>
   </bookViews>
   <sheets>
     <sheet name="car inventory" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'car inventory'!$1:$1</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -963,17 +979,7 @@
     <cellStyle name="Total" xfId="18" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="15" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -986,11 +992,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1008,9 +1014,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1048,7 +1054,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1154,7 +1160,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1296,7 +1302,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1304,23 +1310,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE1BE64A-6E35-46AF-B538-7FFA7D2A357E}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:N67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="7"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="7"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="4" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" customWidth="1"/>
-    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5546875" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.6640625" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1364,7 +1373,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>14</v>
       </c>
@@ -1417,7 +1426,7 @@
         <v>FD06MTGBLA001</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
@@ -1470,7 +1479,7 @@
         <v>FD06MTGWHI002</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
@@ -1523,7 +1532,7 @@
         <v>FD08MTGGRE003</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>23</v>
       </c>
@@ -1576,7 +1585,7 @@
         <v>FD08MTGBLA004</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>25</v>
       </c>
@@ -1629,7 +1638,7 @@
         <v>FD08MTGWHI005</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>119</v>
       </c>
@@ -1682,7 +1691,7 @@
         <v>FD06FCSGRE006</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>27</v>
       </c>
@@ -1735,7 +1744,7 @@
         <v>FD06FCSGRE007</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>28</v>
       </c>
@@ -1788,7 +1797,7 @@
         <v>FD09FCSBLA008</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>30</v>
       </c>
@@ -1841,7 +1850,7 @@
         <v>FD13FCSBLA009</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>31</v>
       </c>
@@ -1894,7 +1903,7 @@
         <v>FD13FCSWHI010</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>33</v>
       </c>
@@ -1947,7 +1956,7 @@
         <v>FD12FCSWHI011</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>35</v>
       </c>
@@ -2000,7 +2009,7 @@
         <v>FD13FCSBLA012</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>37</v>
       </c>
@@ -2053,7 +2062,7 @@
         <v>FD13FCSBLA013</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>120</v>
       </c>
@@ -2106,7 +2115,7 @@
         <v>GM09CMRWHI014</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>40</v>
       </c>
@@ -2159,7 +2168,7 @@
         <v>GM12CMRBLA015</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>42</v>
       </c>
@@ -2212,7 +2221,7 @@
         <v>GM14CMRWHI016</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>44</v>
       </c>
@@ -2265,7 +2274,7 @@
         <v>GM10SLVBLA017</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>46</v>
       </c>
@@ -2318,7 +2327,7 @@
         <v>GM98SLVBLA018</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>47</v>
       </c>
@@ -2371,7 +2380,7 @@
         <v>GM00SLVBLU019</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>49</v>
       </c>
@@ -2424,7 +2433,7 @@
         <v>TY96CAMGRE020</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>51</v>
       </c>
@@ -2477,7 +2486,7 @@
         <v>TY98CAMBLA021</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>53</v>
       </c>
@@ -2530,7 +2539,7 @@
         <v>TY00CAMGRE022</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>54</v>
       </c>
@@ -2583,7 +2592,7 @@
         <v>TY02CAMBLA023</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>55</v>
       </c>
@@ -2636,7 +2645,7 @@
         <v>TY09CAMWHI024</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>56</v>
       </c>
@@ -2689,7 +2698,7 @@
         <v>TY02CORRED025</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>59</v>
       </c>
@@ -2742,7 +2751,7 @@
         <v>TY03CORBLA026</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>60</v>
       </c>
@@ -2795,7 +2804,7 @@
         <v>TY14CORBLU027</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>61</v>
       </c>
@@ -2848,7 +2857,7 @@
         <v>TY12CORBLA028</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>62</v>
       </c>
@@ -2901,7 +2910,7 @@
         <v>TY12CAMBLU029</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>63</v>
       </c>
@@ -2954,7 +2963,7 @@
         <v>HO99CIVWHI030</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>64</v>
       </c>
@@ -3007,7 +3016,7 @@
         <v>HO01CIVBLU031</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>65</v>
       </c>
@@ -3060,7 +3069,7 @@
         <v>HO10CIVBLU032</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>66</v>
       </c>
@@ -3113,7 +3122,7 @@
         <v>HO10CIVBLA033</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>67</v>
       </c>
@@ -3166,7 +3175,7 @@
         <v>HO11CIVBLA034</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>68</v>
       </c>
@@ -3219,7 +3228,7 @@
         <v>HO12CIVBLA035</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>69</v>
       </c>
@@ -3272,7 +3281,7 @@
         <v>HO13CIVBLA036</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>121</v>
       </c>
@@ -3325,7 +3334,7 @@
         <v>HO05ODYWHI037</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>70</v>
       </c>
@@ -3378,7 +3387,7 @@
         <v>HO07ODYBLA038</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>71</v>
       </c>
@@ -3431,7 +3440,7 @@
         <v>HO08ODYWHI039</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>118</v>
       </c>
@@ -3484,7 +3493,7 @@
         <v>HO01ODYBLA040</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>72</v>
       </c>
@@ -3537,7 +3546,7 @@
         <v>HO14ODYBLA041</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>73</v>
       </c>
@@ -3590,7 +3599,7 @@
         <v>CR04PTCBLU042</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>74</v>
       </c>
@@ -3643,7 +3652,7 @@
         <v>CR07PTCGRE043</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>75</v>
       </c>
@@ -3696,7 +3705,7 @@
         <v>CR11PTCBLA044</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>76</v>
       </c>
@@ -3749,7 +3758,7 @@
         <v>CR99CARGRE045</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>77</v>
       </c>
@@ -3802,7 +3811,7 @@
         <v>CR00CARBLA046</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>78</v>
       </c>
@@ -3855,7 +3864,7 @@
         <v>CR04CARWHI047</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>79</v>
       </c>
@@ -3908,7 +3917,7 @@
         <v>CR04CARRED048</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>80</v>
       </c>
@@ -3961,7 +3970,7 @@
         <v>HY11ELABLA049</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>81</v>
       </c>
@@ -4014,7 +4023,7 @@
         <v>HY12ELABLU050</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>82</v>
       </c>
@@ -4067,7 +4076,7 @@
         <v>HY13ELABLA051</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>83</v>
       </c>
@@ -4120,7 +4129,7 @@
         <v>HY13ELABLU052</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B57" s="7" t="s">
         <v>84</v>
       </c>
@@ -4134,7 +4143,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B58" s="7" t="s">
         <v>89</v>
       </c>
@@ -4148,7 +4157,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B59" s="7" t="s">
         <v>88</v>
       </c>
@@ -4162,7 +4171,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B60" s="7" t="s">
         <v>87</v>
       </c>
@@ -4176,7 +4185,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B61" s="7" t="s">
         <v>85</v>
       </c>
@@ -4190,7 +4199,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B62" s="7" t="s">
         <v>86</v>
       </c>
@@ -4204,7 +4213,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D63" s="4" t="s">
         <v>100</v>
       </c>
@@ -4212,7 +4221,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D64" s="4" t="s">
         <v>110</v>
       </c>
@@ -4220,7 +4229,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="65" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D65" s="4" t="s">
         <v>112</v>
       </c>
@@ -4228,7 +4237,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="66" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D66" s="4" t="s">
         <v>114</v>
       </c>
@@ -4236,7 +4245,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="67" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D67" s="4" t="s">
         <v>116</v>
       </c>
@@ -4245,18 +4254,18 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D57:E67">
-    <sortCondition ref="D57:D67"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B57:C62">
+    <sortCondition ref="B57:B62"/>
   </sortState>
   <conditionalFormatting sqref="M2:M53">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Not Covered"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Y"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Not Covered"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="79" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>